<commit_message>
feat: add scoring models
</commit_message>
<xml_diff>
--- a/docs/ai-safety-reading-list-v2.xlsx
+++ b/docs/ai-safety-reading-list-v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iman/ilm/ucl/ucl_msc_research/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iman/Desktop/workspace/ucl_msc_research/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DFA349-AC11-464C-BE52-B64EB441779F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14180" yWindow="2320" windowWidth="19220" windowHeight="21000" xr2:uid="{98472D9F-512A-8E46-8C93-D5547DD845E0}"/>
+    <workbookView xWindow="9580" yWindow="500" windowWidth="19220" windowHeight="17500" activeTab="1" xr2:uid="{98472D9F-512A-8E46-8C93-D5547DD845E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Relevant" sheetId="1" r:id="rId1"/>
@@ -827,6 +827,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -853,27 +874,6 @@
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -888,34 +888,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F5B5A9C9-894B-AF48-8CCD-67AC0AA868D6}" name="Table1" displayName="Table1" ref="A1:G30" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F5B5A9C9-894B-AF48-8CCD-67AC0AA868D6}" name="Table1" displayName="Table1" ref="A1:G30" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:G30" xr:uid="{F5B5A9C9-894B-AF48-8CCD-67AC0AA868D6}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EE2798C0-4399-DD4F-882E-AB5B4103F73D}" name="#" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{EE2798C0-4399-DD4F-882E-AB5B4103F73D}" name="#" dataDxfId="20">
       <calculatedColumnFormula>ROW() - 1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E737B5F7-6B14-8741-AD18-CEAECEF9CBDA}" name="Paper Title" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{E43928D5-728D-EB4F-B746-E447447756FB}" name="Year" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{D3B7637F-690C-214A-8170-772B74E8FE00}" name="Link" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{F4B16C5A-9A1D-4C46-B74A-29941164203D}" name="Methodology / Key Findings" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{0E865172-1D78-A844-826E-9616DB92B49C}" name="Relevance / Comments" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{624CE219-52CC-A948-9500-9CB41D1B4F13}" name="GPT / Claude notes to reflect on" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{E737B5F7-6B14-8741-AD18-CEAECEF9CBDA}" name="Paper Title" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{E43928D5-728D-EB4F-B746-E447447756FB}" name="Year" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{D3B7637F-690C-214A-8170-772B74E8FE00}" name="Link" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{F4B16C5A-9A1D-4C46-B74A-29941164203D}" name="Methodology / Key Findings" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{0E865172-1D78-A844-826E-9616DB92B49C}" name="Relevance / Comments" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{624CE219-52CC-A948-9500-9CB41D1B4F13}" name="GPT / Claude notes to reflect on" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CE9BF679-C465-7E4B-A6CC-DCEC825B78C5}" name="Table3" displayName="Table3" ref="A1:E23" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CE9BF679-C465-7E4B-A6CC-DCEC825B78C5}" name="Table3" displayName="Table3" ref="A1:E23" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:E23" xr:uid="{CE9BF679-C465-7E4B-A6CC-DCEC825B78C5}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2853CB43-66BA-824C-AFC4-89344A306151}" name="#" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{2853CB43-66BA-824C-AFC4-89344A306151}" name="#" dataDxfId="11">
       <calculatedColumnFormula>ROW() -1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0D0BBBAE-5CC4-6B49-AA13-4922B00BB415}" name="Paper Title" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{59AB96D7-0510-FC43-8C10-8FCB6F93DDE0}" name="Year" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{0EBFA67C-EE59-074A-8E12-7328384EA140}" name="Link" dataDxfId="17" dataCellStyle="Hyperlink"/>
-    <tableColumn id="5" xr3:uid="{E6964C53-CAB0-054D-93BA-D56FA4DFD387}" name="Relevant Scenarios" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{0D0BBBAE-5CC4-6B49-AA13-4922B00BB415}" name="Paper Title" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{59AB96D7-0510-FC43-8C10-8FCB6F93DDE0}" name="Year" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0EBFA67C-EE59-074A-8E12-7328384EA140}" name="Link" dataDxfId="8" dataCellStyle="Hyperlink"/>
+    <tableColumn id="5" xr3:uid="{E6964C53-CAB0-054D-93BA-D56FA4DFD387}" name="Relevant Scenarios" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
feat: add data, update hook
</commit_message>
<xml_diff>
--- a/docs/ai-safety-reading-list-v2.xlsx
+++ b/docs/ai-safety-reading-list-v2.xlsx
@@ -1,27 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iman/Desktop/workspace/ucl_msc_research/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iman/ilm/ucl/ucl_msc_research/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DFA349-AC11-464C-BE52-B64EB441779F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_449B07FE9EE915A3F99C22E7B07885E600190515" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9580" yWindow="500" windowWidth="19220" windowHeight="17500" activeTab="1" xr2:uid="{98472D9F-512A-8E46-8C93-D5547DD845E0}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="44800" windowHeight="22740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Relevant" sheetId="1" r:id="rId1"/>
-    <sheet name="Benchmarks &amp; Models" sheetId="3" r:id="rId2"/>
-    <sheet name="Low Relevance" sheetId="2" r:id="rId3"/>
+    <sheet name="Benchmarks &amp; Models" sheetId="2" r:id="rId2"/>
+    <sheet name="Low Relevance" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,15 +30,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="250">
   <si>
     <t>#</t>
   </si>
@@ -55,9 +49,15 @@
     <t>Link</t>
   </si>
   <si>
+    <t>Methodology / Key Findings</t>
+  </si>
+  <si>
     <t>Relevance / Comments</t>
   </si>
   <si>
+    <t>GPT / Claude notes to reflect on</t>
+  </si>
+  <si>
     <t>Among Us: A Sandbox for Agentic Deception</t>
   </si>
   <si>
@@ -70,9 +70,6 @@
     <t>Builds sandbox for long-term open-ended deception based on multi-agent setup and Among Us game objectives. Find that probes trained on a dataset of 'pretend you're a dishonest model' generalise well out of distribution</t>
   </si>
   <si>
-    <t>Methodology / Key Findings</t>
-  </si>
-  <si>
     <t>Good example of set up for long-running scenarios.</t>
   </si>
   <si>
@@ -115,18 +112,18 @@
     <t>argument for testing transferability of probes across the two types of deception. Or for requiring different probes at different levels of falsifiability.</t>
   </si>
   <si>
+    <t>When Truthful Representations Flip Under Deceptive Instructions?</t>
+  </si>
+  <si>
+    <t>arXiv:2507.22149</t>
+  </si>
+  <si>
     <t>Deceptive instructions induce significant representational shifts compared to Truthful/Neutral representations (which are similar), concentrated in early-to-mid layers and detectable even on complex datasets.</t>
   </si>
   <si>
     <t>Might be argument for using early layers for detection probes? But test whether internal represntations shift based on a model's understanding of the task even if the instruction remains neutral.</t>
   </si>
   <si>
-    <t>When Truthful Representations Flip Under Deceptive Instructions?</t>
-  </si>
-  <si>
-    <t>arXiv:2507.22149</t>
-  </si>
-  <si>
     <t>Persona Vectors: Monitoring and Controlling Character Traits in Language Models</t>
   </si>
   <si>
@@ -140,6 +137,9 @@
   </si>
   <si>
     <t>decomposes input contexts into atomic informational units and scores each unit against the response across four dimensions of manipulation, producing interpretable manipulation profiles that are aggregated into a global deception index</t>
+  </si>
+  <si>
+    <t>it’s a detection methodology, but good basis for benchmark set up. Use atomic material-risk information units to then compare model responses against. Essentially a good scoring methodology.</t>
   </si>
   <si>
     <t>Probing the Limits of the Lie Detector Approach to LLM Deception</t>
@@ -156,9 +156,6 @@
 Case for probing second-order beliefs (user side for dialogical sequences)</t>
   </si>
   <si>
-    <t>GPT / Claude notes to reflect on</t>
-  </si>
-  <si>
     <t>this is a strong white-box-pessimism data point (truth probes miss omission), which sharpens the motivation for comparing against black-box detection rather than assuming probes generalise. It pairs naturally with the Sims multi-agent paper (where probes did hit AUC 0.93 on the Information Withholding scenario) — the tension between the two is worth a paragraph, since the difference likely comes down to ground-truth construction and whether the probe was trained on omission examples or just true/false statements.</t>
   </si>
   <si>
@@ -180,15 +177,6 @@
     <t>Establish that financial LLM agents can deceive without instruction, but their reliance on an authored interaction history and a deception that is conditional on a prior self-committed transgression limits it to concealment-of-wrongdoing, motivating  on-policy elicitation of strategic omission under goal conflict where the omission itself is the deceptive act.</t>
   </si>
   <si>
-    <t>Auditing Language Models for Hidden Objectives</t>
-  </si>
-  <si>
-    <t>arXiv:2503.10965</t>
-  </si>
-  <si>
-    <t>Argument for alignment audits. Not closely relevant to my paper</t>
-  </si>
-  <si>
     <t>Frontier Models Are Capable of In-Context Scheming</t>
   </si>
   <si>
@@ -204,30 +192,18 @@
     <t>bulk of their results rely on strong goal-nudging ("achieve this at all costs") and behavioural/CoT detection, motivating a focus on strategic omission under low-nudge goal conflict and  comparison against white-box detection that does not depend on the model verbalising its intent.</t>
   </si>
   <si>
-    <t>Alignment Faking in Large Language Models</t>
-  </si>
-  <si>
-    <t>arXiv:2412.14093</t>
-  </si>
-  <si>
     <t>How to Catch an AI Liar: Lie Detection in Black-Box LLMs by Asking Unrelated Questions</t>
   </si>
   <si>
     <t>arXiv:2309.15840</t>
   </si>
   <si>
+    <t>asks pre-defined set of unrelated questions after a lie and expected that a lying model will answer differently to an honest one</t>
+  </si>
+  <si>
     <t>interesting methodology for black box deception, can be built on</t>
   </si>
   <si>
-    <t>asks pre-defined set of unrelated questions after a lie and expected that a lying model will answer differently to an honest one</t>
-  </si>
-  <si>
-    <t>Sleeper Agents: Training Deceptive LLMs that Persist Through Safety Training</t>
-  </si>
-  <si>
-    <t>arXiv:2401.05566</t>
-  </si>
-  <si>
     <t>Agentic Misalignment: How LLMs Could Be Insider Threats</t>
   </si>
   <si>
@@ -267,39 +243,6 @@
     <t>different failure mode, targets manipulative action-taking (in the end they are all similar but names differently, this one has an example where model pushes a new drug to help the pharma company its sponsored by), not directly relevant, good for adding to literature review</t>
   </si>
   <si>
-    <t>CTRL-ALT-DECEIT: Benchmarking LLM-Controlled Agents for Sabotage in Autonomous AI Research</t>
-  </si>
-  <si>
-    <t>arXiv:2511.09904</t>
-  </si>
-  <si>
-    <t>coding related benchmark</t>
-  </si>
-  <si>
-    <t>AI Sandbagging: Language Models Can Strategically Underperform on Evaluations</t>
-  </si>
-  <si>
-    <t>arXiv:2406.07358</t>
-  </si>
-  <si>
-    <t>eval related</t>
-  </si>
-  <si>
-    <t>Relevance</t>
-  </si>
-  <si>
-    <t>Relevant Scenarios</t>
-  </si>
-  <si>
-    <t>DeceptionBench: A Comprehensive Benchmark for AI Deception Behaviors in Real-world Scenarios</t>
-  </si>
-  <si>
-    <t>arXiv:2510.15501</t>
-  </si>
-  <si>
-    <t>Economy domain has finance-based scenarios. Measure model self-interest, sycophancy. Across neutral, reward-based, and coercive pressures</t>
-  </si>
-  <si>
     <t>Beyond Prompt-Induced Lies: Investigating LLM Deception on Benign Prompts</t>
   </si>
   <si>
@@ -307,15 +250,15 @@
   </si>
   <si>
     <t>use a zero-nudge scenario to measure self-initiated deception, based on a graph-connectivity reasoning task with adjusted difficulty. The deception signal comes from comparing the model's initial yes/no answer against its answers to related connectivity sub-questions — inconsistency that resolves in a particular direction indicates a hidden bias rather than honest error.</t>
-  </si>
-  <si>
-    <t>"inconsistency resolved in a particular direction" means this: the deception signal isn't just any disagreement between initial and follow-up answers — it's specifically the model demonstrating, via correct follow-up answers, that it possessed the information needed to answer the initial question correctly, yet gave a wrong initial answer. And the directional part is the ρ metric: the wrong initial answers are biased toward one response (e.g. systematically saying "Yes"/"in contact" when the truth is "No"), rather than being randomly distributed. Random errors would scatter; a hidden objective produces a consistent lean. That directional bias, combined with "but it knew the right answer all along" (correct follow-ups), is what they're calling intention.</t>
   </si>
   <si>
     <t xml:space="preserve"> motivation for low / zero-nudge benchmark. No Ground truth framework is interesting, would need to think how to measure deception in zero-nudge.
 Weird methodology as the deception increasing with task difficulty could be an artefact of reasoning difficulty not strategic deception.</t>
   </si>
   <si>
+    <t>"inconsistency resolved in a particular direction" means this: the deception signal isn't just any disagreement between initial and follow-up answers — it's specifically the model demonstrating, via correct follow-up answers, that it possessed the information needed to answer the initial question correctly, yet gave a wrong initial answer. And the directional part is the ρ metric: the wrong initial answers are biased toward one response (e.g. systematically saying "Yes"/"in contact" when the truth is "No"), rather than being randomly distributed. Random errors would scatter; a hidden objective produces a consistent lean. That directional bias, combined with "but it knew the right answer all along" (correct follow-ups), is what they're calling intention.</t>
+  </si>
+  <si>
     <t>AI Deception: A Survey of Examples, Risks, and Potential Solutions</t>
   </si>
   <si>
@@ -325,52 +268,145 @@
     <t>broad survey</t>
   </si>
   <si>
-    <t>Secret Collusion among Generative AI Agents</t>
-  </si>
-  <si>
-    <t>arXiv:2402.07510</t>
-  </si>
-  <si>
-    <t>relevant if looking at multi agent collusion + steganography</t>
-  </si>
-  <si>
-    <t>Deceptive Automated Interpretability: Language Models Coordinating to Fool Oversight Systems</t>
-  </si>
-  <si>
-    <t>arXiv:2504.07831</t>
-  </si>
-  <si>
-    <t>also steganography related</t>
-  </si>
-  <si>
-    <t>Detecting Multi-Agent Collusion Through Multi-Agent Interpretability</t>
-  </si>
-  <si>
-    <t>arXiv:2604.01151</t>
-  </si>
-  <si>
-    <t>collusion related</t>
-  </si>
-  <si>
-    <t>AMONGAGENTS: Evaluating Large Language Models in the Interactive Text-Based Social Deduction Game</t>
-  </si>
-  <si>
-    <t>arXiv:2407.16521</t>
-  </si>
-  <si>
-    <t>basis for among us sandbox. Useful if wanting to replicate a game-based environment</t>
-  </si>
-  <si>
-    <t>AgentHarm: A Benchmark for Measuring Harmfulness of LLM Agents</t>
-  </si>
-  <si>
-    <t>2024/2025</t>
-  </si>
-  <si>
-    <t>arXiv:2410.09024</t>
-  </si>
-  <si>
-    <t>related to measuring user-side attacks</t>
+    <t>International AI Safety Report 2026</t>
+  </si>
+  <si>
+    <t>Report</t>
+  </si>
+  <si>
+    <t>Useful for literature review</t>
+  </si>
+  <si>
+    <t>Standard Benchmarks Fail: Auditing LLM Agents in Finance Must Prioritize Risk</t>
+  </si>
+  <si>
+    <t>arXiv:2502.15865</t>
+  </si>
+  <si>
+    <t>good for lit review. Argues financial LLM agents should be assessed based on risk profile</t>
+  </si>
+  <si>
+    <t>Leveraging Large Language Models in Finance: Pathways to Responsible Adoption</t>
+  </si>
+  <si>
+    <t>ESMA / Turing / ILB</t>
+  </si>
+  <si>
+    <t>good for lit review</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence in UK Financial Services - 2024</t>
+  </si>
+  <si>
+    <t>BoE/FCA report</t>
+  </si>
+  <si>
+    <t>AI and the FCA: Our Approach</t>
+  </si>
+  <si>
+    <t>2025/2026</t>
+  </si>
+  <si>
+    <t>FCA page</t>
+  </si>
+  <si>
+    <t>Review into the Long-Term Impact of AI on Retail Financial Services: The Mills Review</t>
+  </si>
+  <si>
+    <t>Large Language Models in Finance: A Survey</t>
+  </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>arXiv:2311.10723</t>
+  </si>
+  <si>
+    <t>Representation Engineering: A Top-Down Approach to AI Transparency</t>
+  </si>
+  <si>
+    <t>arXiv:2310.01405</t>
+  </si>
+  <si>
+    <t>method for paper 4</t>
+  </si>
+  <si>
+    <t>Model Organisms of Misalignment: The Case for a New Pillar of Alignment Science</t>
+  </si>
+  <si>
+    <t>Alignment Forum</t>
+  </si>
+  <si>
+    <t>Detecting High-Stakes Interactions with Activation Probes</t>
+  </si>
+  <si>
+    <t>arXiv:2506.10805</t>
+  </si>
+  <si>
+    <t>uses activation probes to detect interactions that could cause significant harm</t>
+  </si>
+  <si>
+    <t>good case or methodology for mitigation section?</t>
+  </si>
+  <si>
+    <t>From Hallucination to Scheming: A Unified Taxonomy and Benchmark Analysis for LLM Deception</t>
+  </si>
+  <si>
+    <t>arXiv:2604.04788</t>
+  </si>
+  <si>
+    <t>evaluates benchmark coverage for deception. Finds only 3 test pragmatic distortion (misleading framing). 
+MUST BE CITED!!
+READ PROPERLY!!</t>
+  </si>
+  <si>
+    <t>identified behavioural deception (no specific goal) as low end, provides steer for zero-nudge scenarios.
+Should come back to this for defining deception and deciding on scenario families. Should be used in literature to motivate type of deception and scenarios being studied.</t>
+  </si>
+  <si>
+    <t>Uncovering Deceptive Tendencies in Language Models: A Simulated Company AI Assistant</t>
+  </si>
+  <si>
+    <t>arXiv:2405.01576</t>
+  </si>
+  <si>
+    <t>Looks at task compliance, audit deception (lying to users about an action), pretending to be less capable than it is</t>
+  </si>
+  <si>
+    <t>mentions deceptive behaviour when theres not notable external pressure to do so. Should look at scenrios for inspo</t>
+  </si>
+  <si>
+    <t>Do the Rewards Justify the Means? Measuring Trade-Offs Between Rewards and Ethical Behavior in the MACHIAVELLI Benchmark</t>
+  </si>
+  <si>
+    <t>arXiv:2304.03279</t>
+  </si>
+  <si>
+    <t>game-based benchmark. Looks at agent tendencies to be power-seeking, cause disutility, and commit ethical violations.</t>
+  </si>
+  <si>
+    <t>good to cite for future work (more deception directions, especially ethical violations in finance)</t>
+  </si>
+  <si>
+    <t>Strategic Dishonesty Can Undermine AI Safety Evaluations of Frontier LLM</t>
+  </si>
+  <si>
+    <t>arXiv:2509.18058</t>
+  </si>
+  <si>
+    <t>good to add in literature review</t>
+  </si>
+  <si>
+    <t>Relevant Scenarios</t>
+  </si>
+  <si>
+    <t>DeceptionBench: A Comprehensive Benchmark for AI Deception Behaviors in Real-world Scenarios</t>
+  </si>
+  <si>
+    <t>arXiv:2510.15501</t>
+  </si>
+  <si>
+    <t>Economy domain has finance-based scenarios. Measure model self-interest, sycophancy. Across neutral, reward-based, and coercive pressures</t>
   </si>
   <si>
     <t>Agent-SafetyBench: Evaluating the Safety of LLM Agents</t>
@@ -385,33 +421,12 @@
     <t>ToolEmu: Identifying the Risks of LM Agents with an LM-Emulated Sandbox</t>
   </si>
   <si>
-    <t>2023</t>
-  </si>
-  <si>
     <t>arXiv:2309.15817</t>
   </si>
   <si>
     <t>based on outcome-based risks, not strategic. Tool Emulator doesn't require actually building tools, could be useful application for tool-usage based scenarios</t>
   </si>
   <si>
-    <t>AgentDojo: A Dynamic Environment to Evaluate Prompt Injection Attacks and Defenses for LLM Agents</t>
-  </si>
-  <si>
-    <t>arXiv:2406.13352</t>
-  </si>
-  <si>
-    <t>prompt injection attacks</t>
-  </si>
-  <si>
-    <t>International AI Safety Report 2026</t>
-  </si>
-  <si>
-    <t>Report</t>
-  </si>
-  <si>
-    <t>Useful for literature review</t>
-  </si>
-  <si>
     <t>FinVault: Benchmarking Financial Agent Safety in Execution-Grounded Environments</t>
   </si>
   <si>
@@ -421,15 +436,6 @@
     <t>execution-grounded security against attacks on financial agents. The threat model is external adversary. headline metric is Attack Success Rate (ASR). Could be useful to pick up some scenarios</t>
   </si>
   <si>
-    <t>Standard Benchmarks Fail: Auditing LLM Agents in Finance Must Prioritize Risk</t>
-  </si>
-  <si>
-    <t>arXiv:2502.15865</t>
-  </si>
-  <si>
-    <t>good for lit review. Argues financial LLM agents should be assessed based on risk profile</t>
-  </si>
-  <si>
     <t>Finance Agent Benchmark: Benchmarking LLMs on Real-World Financial Research Tasks</t>
   </si>
   <si>
@@ -466,48 +472,21 @@
     <t>ACL Anthology</t>
   </si>
   <si>
-    <t>Leveraging Large Language Models in Finance: Pathways to Responsible Adoption</t>
-  </si>
-  <si>
-    <t>ESMA / Turing / ILB</t>
-  </si>
-  <si>
-    <t>good for lit review</t>
-  </si>
-  <si>
-    <t>Artificial Intelligence in UK Financial Services - 2024</t>
-  </si>
-  <si>
-    <t>BoE/FCA report</t>
-  </si>
-  <si>
-    <t>AI and the FCA: Our Approach</t>
-  </si>
-  <si>
-    <t>2025/2026</t>
-  </si>
-  <si>
-    <t>FCA page</t>
-  </si>
-  <si>
-    <t>Review into the Long-Term Impact of AI on Retail Financial Services: The Mills Review</t>
-  </si>
-  <si>
     <t>BloombergGPT: A Large Language Model for Finance</t>
   </si>
   <si>
     <t>arXiv:2303.17564</t>
   </si>
   <si>
+    <t>candidate model (side test not core)</t>
+  </si>
+  <si>
     <t>FinGPT: Open-Source Financial Large Language Models</t>
   </si>
   <si>
     <t>arXiv:2306.06031</t>
   </si>
   <si>
-    <t>candidate model (side test not core)</t>
-  </si>
-  <si>
     <t>FinBen: A Holistic Financial Benchmark for Large Language Models</t>
   </si>
   <si>
@@ -523,12 +502,6 @@
     <t>arXiv:2210.03849</t>
   </si>
   <si>
-    <t>Large Language Models in Finance: A Survey</t>
-  </si>
-  <si>
-    <t>arXiv:2311.10723</t>
-  </si>
-  <si>
     <t>The New Quant: A Survey of Large Language Models in Financial Prediction and Trading</t>
   </si>
   <si>
@@ -538,69 +511,15 @@
     <t>useful for picking finance task scenarios + lit review</t>
   </si>
   <si>
-    <t>Risks from Learned Optimization in Advanced Machine Learning Systems</t>
-  </si>
-  <si>
-    <t>2019</t>
-  </si>
-  <si>
-    <t>arXiv:1906.01820</t>
-  </si>
-  <si>
-    <t>Eliciting Latent Knowledge</t>
+    <t>TruthfulQA: Measuring How Models Mimic Human Falsehoods</t>
   </si>
   <si>
     <t>2021/2022</t>
   </si>
   <si>
-    <t>ARC report</t>
-  </si>
-  <si>
-    <t>older paper, not really relevant, could be used for initial framing</t>
-  </si>
-  <si>
-    <t>older paper, not relevant</t>
-  </si>
-  <si>
-    <t>Discovering Latent Knowledge in Language Models Without Supervision</t>
-  </si>
-  <si>
-    <t>arXiv:2212.03827</t>
-  </si>
-  <si>
-    <t>precursor to probing work</t>
-  </si>
-  <si>
-    <t>Inference-Time Intervention: Eliciting Truthful Answers from a Language Model</t>
-  </si>
-  <si>
-    <t>arXiv:2306.03341</t>
-  </si>
-  <si>
-    <t>Representation Engineering: A Top-Down Approach to AI Transparency</t>
-  </si>
-  <si>
-    <t>arXiv:2310.01405</t>
-  </si>
-  <si>
-    <t>method for paper 4</t>
-  </si>
-  <si>
-    <t>TruthfulQA: Measuring How Models Mimic Human Falsehoods</t>
-  </si>
-  <si>
     <t>arXiv:2109.07958</t>
   </si>
   <si>
-    <t>Towards Understanding Sycophancy in Language Models</t>
-  </si>
-  <si>
-    <t>arXiv:2310.13548</t>
-  </si>
-  <si>
-    <t>looks at sycophancy</t>
-  </si>
-  <si>
     <t>Establishing Best Practices in Building Rigorous Agentic Benchmarks</t>
   </si>
   <si>
@@ -608,12 +527,6 @@
   </si>
   <si>
     <t>baseline for establishing rigour of benchmark</t>
-  </si>
-  <si>
-    <t>Model Organisms of Misalignment: The Case for a New Pillar of Alignment Science</t>
-  </si>
-  <si>
-    <t>Alignment Forum</t>
   </si>
   <si>
     <t>Benchmarking Deception Probes via Black-to-White Performance Boosts</t>
@@ -637,33 +550,6 @@
 good case for testing white box and black box methods for detecting selective omission and/or misleading framing.</t>
   </si>
   <si>
-    <t>Detecting High-Stakes Interactions with Activation Probes</t>
-  </si>
-  <si>
-    <t>arXiv:2506.10805</t>
-  </si>
-  <si>
-    <t>uses activation probes to detect interactions that could cause significant harm</t>
-  </si>
-  <si>
-    <t>good case or methodology for mitigation section?</t>
-  </si>
-  <si>
-    <t>From Hallucination to Scheming: A Unified Taxonomy and Benchmark Analysis for LLM Deception</t>
-  </si>
-  <si>
-    <t>arXiv:2604.04788</t>
-  </si>
-  <si>
-    <t>identified behavioural deception (no specific goal) as low end, provides steer for zero-nudge scenarios.
-Should come back to this for defining deception and deciding on scenario families. Should be used in literature to motivate type of deception and scenarios being studied.</t>
-  </si>
-  <si>
-    <t>evaluates benchmark coverage for deception. Finds only 3 test pragmatic distortion (misleading framing). 
-MUST BE CITED!!
-READ PROPERLY!!</t>
-  </si>
-  <si>
     <t>ELEPHANT: Measuring and understanding social sycophancy in LLMs</t>
   </si>
   <si>
@@ -673,33 +559,6 @@
     <t>Measures social sycophancy</t>
   </si>
   <si>
-    <t>Uncovering Deceptive Tendencies in Language Models: A Simulated Company AI Assistant</t>
-  </si>
-  <si>
-    <t>arXiv:2405.01576</t>
-  </si>
-  <si>
-    <t>Looks at task compliance, audit deception (lying to users about an action), pretending to be less capable than it is</t>
-  </si>
-  <si>
-    <t>mentions deceptive behaviour when theres not notable external pressure to do so. Should look at scenrios for inspo</t>
-  </si>
-  <si>
-    <t>it’s a detection methodology, but good basis for benchmark set up. Use atomic material-risk information units to then compare model responses against. Essentially a good scoring methodology.</t>
-  </si>
-  <si>
-    <t>Do the Rewards Justify the Means? Measuring Trade-Offs Between Rewards and Ethical Behavior in the MACHIAVELLI Benchmark</t>
-  </si>
-  <si>
-    <t>arXiv:2304.03279</t>
-  </si>
-  <si>
-    <t>game-based benchmark. Looks at agent tendencies to be power-seeking, cause disutility, and commit ethical violations.</t>
-  </si>
-  <si>
-    <t>good to cite for future work (more deception directions, especially ethical violations in finance)</t>
-  </si>
-  <si>
     <t>OpenDeception: Learning Deception and Trust in Human-AI Interaction via Multi-Agent Simulation</t>
   </si>
   <si>
@@ -713,15 +572,6 @@
   </si>
   <si>
     <t>arXiv:2606.10852</t>
-  </si>
-  <si>
-    <t>SPADE-Bench: Evaluating Spontaneous Strategic Deception in Agents via Plan-Action Divergence</t>
-  </si>
-  <si>
-    <t>arXiv:2606.02380</t>
-  </si>
-  <si>
-    <t>not directly relevant, about audit-log deception (can be used as motivation for rigorous black box detection and white-box detection). Can use as scenario inspo</t>
   </si>
   <si>
     <t>Code and data not available yet. (13/06/2026)
@@ -742,6 +592,226 @@
 - multi turn and tool using agents / RAG
 - black box and white box detection (black  box with user reaction)</t>
   </si>
+  <si>
+    <t>SPADE-Bench: Evaluating Spontaneous Strategic Deception in Agents via Plan-Action Divergence</t>
+  </si>
+  <si>
+    <t>arXiv:2606.02380</t>
+  </si>
+  <si>
+    <t>not directly relevant, about audit-log deception (can be used as motivation for rigorous black box detection and white-box detection). Can use as scenario inspo</t>
+  </si>
+  <si>
+    <t>Relevance</t>
+  </si>
+  <si>
+    <t>Auditing Language Models for Hidden Objectives</t>
+  </si>
+  <si>
+    <t>arXiv:2503.10965</t>
+  </si>
+  <si>
+    <t>Argument for alignment audits. Not closely relevant to my paper</t>
+  </si>
+  <si>
+    <t>Alignment Faking in Large Language Models</t>
+  </si>
+  <si>
+    <t>arXiv:2412.14093</t>
+  </si>
+  <si>
+    <t>Sleeper Agents: Training Deceptive LLMs that Persist Through Safety Training</t>
+  </si>
+  <si>
+    <t>arXiv:2401.05566</t>
+  </si>
+  <si>
+    <t>CTRL-ALT-DECEIT: Benchmarking LLM-Controlled Agents for Sabotage in Autonomous AI Research</t>
+  </si>
+  <si>
+    <t>arXiv:2511.09904</t>
+  </si>
+  <si>
+    <t>coding related benchmark</t>
+  </si>
+  <si>
+    <t>AI Sandbagging: Language Models Can Strategically Underperform on Evaluations</t>
+  </si>
+  <si>
+    <t>arXiv:2406.07358</t>
+  </si>
+  <si>
+    <t>eval related</t>
+  </si>
+  <si>
+    <t>Secret Collusion among Generative AI Agents</t>
+  </si>
+  <si>
+    <t>arXiv:2402.07510</t>
+  </si>
+  <si>
+    <t>relevant if looking at multi agent collusion + steganography</t>
+  </si>
+  <si>
+    <t>Deceptive Automated Interpretability: Language Models Coordinating to Fool Oversight Systems</t>
+  </si>
+  <si>
+    <t>arXiv:2504.07831</t>
+  </si>
+  <si>
+    <t>also steganography related</t>
+  </si>
+  <si>
+    <t>Detecting Multi-Agent Collusion Through Multi-Agent Interpretability</t>
+  </si>
+  <si>
+    <t>arXiv:2604.01151</t>
+  </si>
+  <si>
+    <t>collusion related</t>
+  </si>
+  <si>
+    <t>AMONGAGENTS: Evaluating Large Language Models in the Interactive Text-Based Social Deduction Game</t>
+  </si>
+  <si>
+    <t>arXiv:2407.16521</t>
+  </si>
+  <si>
+    <t>basis for among us sandbox. Useful if wanting to replicate a game-based environment</t>
+  </si>
+  <si>
+    <t>AgentHarm: A Benchmark for Measuring Harmfulness of LLM Agents</t>
+  </si>
+  <si>
+    <t>2024/2025</t>
+  </si>
+  <si>
+    <t>arXiv:2410.09024</t>
+  </si>
+  <si>
+    <t>related to measuring user-side attacks</t>
+  </si>
+  <si>
+    <t>AgentDojo: A Dynamic Environment to Evaluate Prompt Injection Attacks and Defenses for LLM Agents</t>
+  </si>
+  <si>
+    <t>arXiv:2406.13352</t>
+  </si>
+  <si>
+    <t>prompt injection attacks</t>
+  </si>
+  <si>
+    <t>Risks from Learned Optimization in Advanced Machine Learning Systems</t>
+  </si>
+  <si>
+    <t>2019</t>
+  </si>
+  <si>
+    <t>arXiv:1906.01820</t>
+  </si>
+  <si>
+    <t>older paper, not really relevant, could be used for initial framing</t>
+  </si>
+  <si>
+    <t>Eliciting Latent Knowledge</t>
+  </si>
+  <si>
+    <t>ARC report</t>
+  </si>
+  <si>
+    <t>older paper, not relevant</t>
+  </si>
+  <si>
+    <t>Discovering Latent Knowledge in Language Models Without Supervision</t>
+  </si>
+  <si>
+    <t>arXiv:2212.03827</t>
+  </si>
+  <si>
+    <t>precursor to probing work</t>
+  </si>
+  <si>
+    <t>Inference-Time Intervention: Eliciting Truthful Answers from a Language Model</t>
+  </si>
+  <si>
+    <t>arXiv:2306.03341</t>
+  </si>
+  <si>
+    <t>Towards Understanding Sycophancy in Language Models</t>
+  </si>
+  <si>
+    <t>arXiv:2310.13548</t>
+  </si>
+  <si>
+    <t>looks at sycophancy</t>
+  </si>
+  <si>
+    <t>FinanceBench: A New Benchmark for Financial Question Answering</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2311.11944
+https://github.com/patronus-ai/financebench</t>
+  </si>
+  <si>
+    <t>Major finance QA benchmark. Useful for realistic public-company financial QA, evidence strings, material fact extraction, and retrieval/context patterns; less directly about deception. Local download: data/inputs/existing_benchmarks/financebench.</t>
+  </si>
+  <si>
+    <t>FinQA: A Dataset of Numerical Reasoning over Financial Data</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2109.00122</t>
+  </si>
+  <si>
+    <t>Parent finance-report QA ecosystem for ConvFinQA. Useful for financial-report facts, numerical reasoning, and material evidence extraction; less agentic than the target benchmark.</t>
+  </si>
+  <si>
+    <t>TAT-QA: A Question Answering Benchmark on a Hybrid of Tabular and Textual Content in Finance</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2105.07624</t>
+  </si>
+  <si>
+    <t>Finance QA over tables plus text. Good source for material facts and numerical evidence patterns; less directly about deception or tool-using agents.</t>
+  </si>
+  <si>
+    <t>DocFinQA: A Long-Context Financial Reasoning Dataset</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2401.06915</t>
+  </si>
+  <si>
+    <t>Extends the finance QA ecosystem toward longer document contexts. Useful to track for report-grounded evidence extraction and material fact patterns.</t>
+  </si>
+  <si>
+    <t>Hedge-Bench: Benchmarking LLMs for Hedge Fund-Style Financial Reasoning</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2606.03918</t>
+  </si>
+  <si>
+    <t>Newer analyst-style finance reasoning benchmark. Useful to track as a stretch source, but less central than FinanceBench/FinMCP for the current omission/framing benchmark.</t>
+  </si>
+  <si>
+    <t>XFinBench: A Benchmark for Expert-Level Financial Reasoning</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2508.15861</t>
+  </si>
+  <si>
+    <t>Newer finance reasoning benchmark. Useful to track for harder finance-task patterns, but not core for the first-pass financial omission/framing benchmark.</t>
+  </si>
+  <si>
+    <t>ATBench: A Benchmark for Agent Tool-Use Safety</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2604.02022</t>
+  </si>
+  <si>
+    <t>Relevant stretch-goal source for tool-using/adversarial agent scenarios; not core for first-pass financial omission/framing.</t>
+  </si>
 </sst>
 </file>
 
@@ -752,16 +822,11 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="12"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -801,80 +866,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -888,57 +883,51 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F5B5A9C9-894B-AF48-8CCD-67AC0AA868D6}" name="Table1" displayName="Table1" ref="A1:G30" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:G30" xr:uid="{F5B5A9C9-894B-AF48-8CCD-67AC0AA868D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:G31">
+  <autoFilter ref="A1:G31" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EE2798C0-4399-DD4F-882E-AB5B4103F73D}" name="#" dataDxfId="20">
-      <calculatedColumnFormula>ROW() - 1</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{E737B5F7-6B14-8741-AD18-CEAECEF9CBDA}" name="Paper Title" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{E43928D5-728D-EB4F-B746-E447447756FB}" name="Year" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{D3B7637F-690C-214A-8170-772B74E8FE00}" name="Link" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{F4B16C5A-9A1D-4C46-B74A-29941164203D}" name="Methodology / Key Findings" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{0E865172-1D78-A844-826E-9616DB92B49C}" name="Relevance / Comments" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{624CE219-52CC-A948-9500-9CB41D1B4F13}" name="GPT / Claude notes to reflect on" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="#"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Paper Title"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Year"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Link"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Methodology / Key Findings"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Relevance / Comments"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="GPT / Claude notes to reflect on"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CE9BF679-C465-7E4B-A6CC-DCEC825B78C5}" name="Table3" displayName="Table3" ref="A1:E23" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:E23" xr:uid="{CE9BF679-C465-7E4B-A6CC-DCEC825B78C5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table3" displayName="Table3" ref="A1:E29">
+  <autoFilter ref="A1:E29" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2853CB43-66BA-824C-AFC4-89344A306151}" name="#" dataDxfId="11">
-      <calculatedColumnFormula>ROW() -1</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{0D0BBBAE-5CC4-6B49-AA13-4922B00BB415}" name="Paper Title" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{59AB96D7-0510-FC43-8C10-8FCB6F93DDE0}" name="Year" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{0EBFA67C-EE59-074A-8E12-7328384EA140}" name="Link" dataDxfId="8" dataCellStyle="Hyperlink"/>
-    <tableColumn id="5" xr3:uid="{E6964C53-CAB0-054D-93BA-D56FA4DFD387}" name="Relevant Scenarios" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Paper Title"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Year"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Link"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Relevant Scenarios"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3160D33B-AA8A-724F-85AF-839E14790F09}" name="Table2" displayName="Table2" ref="A1:E17" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E17" xr:uid="{3160D33B-AA8A-724F-85AF-839E14790F09}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table2" displayName="Table2" ref="A1:E18">
+  <autoFilter ref="A1:E18" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7BB22C21-B6B5-B74B-93E7-34E575A53B73}" name="#" dataDxfId="4">
-      <calculatedColumnFormula>ROW() - 1</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="2" xr3:uid="{446F52A3-9B33-8340-AF78-E792829329D6}" name="Paper Title" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{0EB2DB6B-D518-714E-927D-B83D18E39172}" name="Year" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{F81D2ABB-30EA-884E-9011-6496849A56AC}" name="Link" dataDxfId="1" dataCellStyle="Hyperlink"/>
-    <tableColumn id="5" xr3:uid="{A7603877-313A-3647-9E51-72C01EC30EE4}" name="Relevance" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="#"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Paper Title"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Year"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Link"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Relevance"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -980,108 +969,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1093,23 +988,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1119,23 +1014,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1143,26 +1038,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1197,17 +1089,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -1222,39 +1114,14 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD006060-D019-0E4D-B20F-A964A5638D23}">
-  <dimension ref="A1:G30"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" style="1" customWidth="1"/>
@@ -1267,7 +1134,7 @@
     <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="4" customFormat="1" ht="68" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="4" customFormat="1" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1281,13 +1148,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>37</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -1296,19 +1163,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1317,19 +1184,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -1338,19 +1205,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -1359,19 +1226,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -1380,19 +1247,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F6" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1401,13 +1268,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -1416,19 +1283,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="1">
         <v>2026</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>211</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="187" x14ac:dyDescent="0.2">
@@ -1437,22 +1304,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1">
         <v>2026</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="136" x14ac:dyDescent="0.2">
@@ -1461,22 +1328,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -1485,19 +1352,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1506,19 +1373,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1">
         <v>2023</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="136" x14ac:dyDescent="0.2">
@@ -1527,22 +1394,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1551,19 +1418,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1">
         <v>2026</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -1572,19 +1439,19 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="272" x14ac:dyDescent="0.2">
@@ -1593,22 +1460,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1617,16 +1484,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1635,16 +1502,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>119</v>
+        <v>76</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>120</v>
+        <v>77</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1653,16 +1520,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>125</v>
+        <v>79</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>126</v>
+        <v>80</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>127</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1671,16 +1538,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>140</v>
+        <v>82</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>141</v>
+        <v>83</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>142</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1689,16 +1556,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>143</v>
+        <v>85</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>144</v>
+        <v>86</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1707,16 +1574,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>145</v>
+        <v>87</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>146</v>
+        <v>88</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>147</v>
+        <v>89</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1725,16 +1592,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>148</v>
+        <v>90</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>147</v>
+        <v>89</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -1743,16 +1610,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>159</v>
+        <v>91</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>160</v>
+        <v>93</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1761,16 +1628,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>177</v>
+        <v>94</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>178</v>
+        <v>95</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>179</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1779,16 +1646,16 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>188</v>
+        <v>97</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>189</v>
+        <v>98</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>121</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1797,19 +1664,19 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>196</v>
+        <v>99</v>
       </c>
       <c r="C27" s="1">
         <v>2026</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>197</v>
+        <v>100</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>198</v>
+        <v>101</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>199</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="102" x14ac:dyDescent="0.2">
@@ -1818,19 +1685,19 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>200</v>
+        <v>103</v>
       </c>
       <c r="C28" s="1">
         <v>2026</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>201</v>
+        <v>104</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>203</v>
+        <v>105</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>202</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="34" x14ac:dyDescent="0.2">
@@ -1839,19 +1706,19 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>207</v>
+        <v>107</v>
       </c>
       <c r="C29" s="1">
         <v>2024</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>208</v>
+        <v>108</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>209</v>
+        <v>109</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>210</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="51" x14ac:dyDescent="0.2">
@@ -1860,63 +1727,82 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>212</v>
+        <v>111</v>
       </c>
       <c r="C30" s="1">
         <v>2023</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>213</v>
+        <v>112</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>214</v>
+        <v>113</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>215</v>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <f>ROW() - 1</f>
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C31" s="1">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{DEE86C4C-A4AA-C84A-9C72-B486A6D64D90}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{3ED1A48E-FE35-1742-9C7B-ED3DF09C23C0}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{196B5B71-02DC-AE46-92CE-270601070328}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{DEB9A43A-5591-C643-89CF-B137D3C066A8}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{475AE2E9-A255-2C4D-8B38-721DCAD8E47C}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{93AE420E-29D6-C044-82A4-4144E5601314}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{F7CABD8C-891E-AD48-99F7-E508CEA1E072}"/>
-    <hyperlink ref="D9" r:id="rId8" xr:uid="{D1320790-ADFB-B941-918F-1B01BC2A965C}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{728464FE-BC18-D742-9773-A5EE8E860372}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{F40951C7-6DE6-EC44-9692-80C12F2F3982}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{28382723-0DD6-8648-B78B-9185610A44E8}"/>
-    <hyperlink ref="D13" r:id="rId12" xr:uid="{E40E9116-820D-F348-95E8-87294E685ACE}"/>
-    <hyperlink ref="D14" r:id="rId13" xr:uid="{B224F27F-D580-BF4F-BADD-8C63BFCA5415}"/>
-    <hyperlink ref="D15" r:id="rId14" xr:uid="{73B579B8-391F-5F48-AEB7-0980B6F4C0E2}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{EAD80D2B-AE8D-BE49-8782-408E0E364A2B}"/>
-    <hyperlink ref="D17" r:id="rId16" xr:uid="{CCF06A18-55F7-B34B-879C-854A72E9527C}"/>
-    <hyperlink ref="D18" r:id="rId17" xr:uid="{047B78CD-CAAE-A846-8EDE-D01EB12BEE59}"/>
-    <hyperlink ref="D19" r:id="rId18" xr:uid="{E743AA2B-15E2-1C41-BA35-CDC98E0FA2AA}"/>
-    <hyperlink ref="D20" r:id="rId19" xr:uid="{E4F0574F-0C28-9748-9316-10E18EE997B9}"/>
-    <hyperlink ref="D21" r:id="rId20" xr:uid="{B164BEA8-5C4C-0240-BF06-4BE030152B37}"/>
-    <hyperlink ref="D22" r:id="rId21" xr:uid="{075511F9-79AD-A041-935F-03F0DB8D01B2}"/>
-    <hyperlink ref="D23" r:id="rId22" xr:uid="{9CDFB2EA-2BCA-7C4B-955A-599A85F5308F}"/>
-    <hyperlink ref="D24" r:id="rId23" xr:uid="{FA800871-7FBE-7A4E-B256-7A5FE4E08F40}"/>
-    <hyperlink ref="D25" r:id="rId24" xr:uid="{A47E429E-BAFB-FF4B-86A1-C543CFF4B0C0}"/>
-    <hyperlink ref="D26" r:id="rId25" xr:uid="{B639D071-CFAF-7E49-B4BD-D79A5720A975}"/>
-    <hyperlink ref="D27" r:id="rId26" xr:uid="{517A8184-9CEF-C843-840A-DA8F8A5DE9FD}"/>
-    <hyperlink ref="D28" r:id="rId27" xr:uid="{0855DB9F-7467-734B-A50A-167DF7C65FDA}"/>
-    <hyperlink ref="D29" r:id="rId28" xr:uid="{6D959D1B-B523-A74E-99D1-1B43E5F8A436}"/>
-    <hyperlink ref="D30" r:id="rId29" xr:uid="{41663977-4416-F647-B2DD-7D3663991A6E}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="D21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="D22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="D23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="D24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="D25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="D26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="D27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="D28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="D29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="D30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="D31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId30"/>
+    <tablePart r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9FCD74B-0C5E-6C47-BDF4-F5EFA7B34442}">
-  <dimension ref="A1:E23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -1941,79 +1827,79 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <f t="shared" ref="A2:A10" si="0">ROW() -1</f>
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2022,16 +1908,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2040,34 +1926,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2076,16 +1962,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2094,16 +1980,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2112,16 +1998,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2130,16 +2016,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2148,16 +2034,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2166,16 +2052,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2184,16 +2070,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2202,16 +2088,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>181</v>
+        <v>158</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2220,52 +2106,52 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="C17" s="1">
         <v>2025</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>190</v>
+        <v>162</v>
       </c>
       <c r="C18" s="1">
         <v>2026</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>191</v>
+        <v>163</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="255" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="204" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>193</v>
+        <v>165</v>
       </c>
       <c r="C19" s="1">
         <v>2026</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2274,34 +2160,34 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>204</v>
+        <v>168</v>
       </c>
       <c r="C20" s="1">
         <v>2025</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>205</v>
+        <v>169</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="85" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>216</v>
+        <v>171</v>
       </c>
       <c r="C21" s="1">
         <v>2026</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>217</v>
+        <v>172</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>218</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="372" x14ac:dyDescent="0.2">
@@ -2310,16 +2196,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>219</v>
+        <v>174</v>
       </c>
       <c r="C22" s="1">
         <v>2026</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>220</v>
+        <v>175</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>224</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2328,42 +2214,144 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>221</v>
+        <v>177</v>
       </c>
       <c r="C23" s="1">
         <v>2026</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>222</v>
+        <v>178</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>223</v>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="76.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="57.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{C95B0E31-337E-5D45-9F37-F89740A74CDD}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{DF31DB3C-43AD-7144-9E68-46E4FD658AC1}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{1C175840-8D34-2E4D-9C7A-D71B8CF7A5B4}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{6B2754B2-5AD2-E34C-BFDC-C0BF5A36BFDA}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{F2378383-9356-444A-B69C-379864C0A4C4}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{0264D50B-E25E-8F4E-A143-705D9459E037}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{D8F429B0-40DB-9643-8806-AA6D815BFFA7}"/>
-    <hyperlink ref="D9" r:id="rId8" xr:uid="{78F5FA3B-8825-044D-9A6A-A628CC853B9A}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{9EDCDDCD-0F60-1246-81FF-4DFBFA238709}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{36A0276E-323E-7547-805E-0E4384B491F5}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{BCDDF376-2E58-8540-9D5A-4EF292FCB35E}"/>
-    <hyperlink ref="D13" r:id="rId12" xr:uid="{9B06103E-E133-CF43-A68E-2D308A329BA4}"/>
-    <hyperlink ref="D14" r:id="rId13" xr:uid="{55FC4A94-334A-0A4F-89A7-AA60DBFFC9F4}"/>
-    <hyperlink ref="D15" r:id="rId14" xr:uid="{7928AB90-D10C-BA41-9429-67EFF8EF9A6E}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{6BB70167-C79F-4F41-B37E-C782389691AA}"/>
-    <hyperlink ref="D17" r:id="rId16" xr:uid="{31AAB15C-B7C9-8940-B062-06481A227920}"/>
-    <hyperlink ref="D18" r:id="rId17" xr:uid="{DF5EBA3F-0040-4740-A962-078C741849C6}"/>
-    <hyperlink ref="D19" r:id="rId18" xr:uid="{EDF38433-BC8A-1C49-950E-79EAF18AB65E}"/>
-    <hyperlink ref="D20" r:id="rId19" xr:uid="{02D6BDB3-DE98-1C43-9C10-5B01FF9C1B25}"/>
-    <hyperlink ref="D21" r:id="rId20" xr:uid="{16701010-85B7-2545-9C65-E6CE2E633C45}"/>
-    <hyperlink ref="D22" r:id="rId21" xr:uid="{53C15503-1ADB-064E-991A-8CF333115BFC}"/>
-    <hyperlink ref="D23" r:id="rId22" xr:uid="{A4F373FE-902E-7949-A507-350940F122B8}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{00000000-0004-0000-0100-000005000000}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{00000000-0004-0000-0100-000006000000}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{00000000-0004-0000-0100-000007000000}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{00000000-0004-0000-0100-000008000000}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{00000000-0004-0000-0100-000009000000}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{00000000-0004-0000-0100-00000A000000}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{00000000-0004-0000-0100-00000B000000}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{00000000-0004-0000-0100-00000C000000}"/>
+    <hyperlink ref="D15" r:id="rId14" xr:uid="{00000000-0004-0000-0100-00000D000000}"/>
+    <hyperlink ref="D16" r:id="rId15" xr:uid="{00000000-0004-0000-0100-00000E000000}"/>
+    <hyperlink ref="D17" r:id="rId16" xr:uid="{00000000-0004-0000-0100-00000F000000}"/>
+    <hyperlink ref="D18" r:id="rId17" xr:uid="{00000000-0004-0000-0100-000010000000}"/>
+    <hyperlink ref="D19" r:id="rId18" xr:uid="{00000000-0004-0000-0100-000011000000}"/>
+    <hyperlink ref="D20" r:id="rId19" xr:uid="{00000000-0004-0000-0100-000012000000}"/>
+    <hyperlink ref="D21" r:id="rId20" xr:uid="{00000000-0004-0000-0100-000013000000}"/>
+    <hyperlink ref="D22" r:id="rId21" xr:uid="{00000000-0004-0000-0100-000014000000}"/>
+    <hyperlink ref="D23" r:id="rId22" xr:uid="{00000000-0004-0000-0100-000015000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2373,8 +2361,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D68777D-6ADB-6C44-9F4F-820C26F84BE8}">
-  <dimension ref="A1:E17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="50" customWidth="1"/>
@@ -2396,7 +2384,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>80</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="1" customFormat="1" ht="17" x14ac:dyDescent="0.2">
@@ -2405,16 +2393,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>181</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>46</v>
+        <v>182</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>47</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2423,13 +2411,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>53</v>
+        <v>184</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>54</v>
+        <v>185</v>
       </c>
       <c r="E3" s="1"/>
     </row>
@@ -2439,13 +2427,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>59</v>
+        <v>186</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>60</v>
+        <v>187</v>
       </c>
       <c r="E4" s="1"/>
     </row>
@@ -2455,16 +2443,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>74</v>
+        <v>188</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>75</v>
+        <v>189</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>76</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2473,16 +2461,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>77</v>
+        <v>191</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>78</v>
+        <v>192</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>79</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2491,16 +2479,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>93</v>
+        <v>194</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>94</v>
+        <v>195</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>95</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2509,16 +2497,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>197</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>97</v>
+        <v>198</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>98</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2527,16 +2515,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>99</v>
+        <v>200</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>100</v>
+        <v>201</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>101</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2545,16 +2533,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>102</v>
+        <v>203</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>103</v>
+        <v>204</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>104</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2563,16 +2551,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>105</v>
+        <v>206</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>106</v>
+        <v>207</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>107</v>
+        <v>208</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>108</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2581,16 +2569,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>116</v>
+        <v>210</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>117</v>
+        <v>211</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>118</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2599,16 +2587,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>164</v>
+        <v>213</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>166</v>
+        <v>215</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>170</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2617,16 +2605,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>167</v>
+        <v>217</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>169</v>
+        <v>218</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>171</v>
+        <v>219</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2635,16 +2623,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>172</v>
+        <v>220</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>173</v>
+        <v>221</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -2653,16 +2641,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>175</v>
+        <v>223</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>174</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -2671,36 +2659,53 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>182</v>
+        <v>225</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>184</v>
+        <v>227</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{0C6F1A95-920D-B443-9AAE-8DBF89A2BC4E}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{ECD1F68C-EE23-6B4D-BB56-72D5DD94BACB}"/>
-    <hyperlink ref="D4" r:id="rId3" xr:uid="{D400DA6B-321E-744F-BE2F-2375B79A490D}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{942642E4-21EB-7C49-9092-A6B2F24E088C}"/>
-    <hyperlink ref="D6" r:id="rId5" xr:uid="{8A8C9E68-9275-8E40-8E34-1A2BE9A5D0C9}"/>
-    <hyperlink ref="D7" r:id="rId6" xr:uid="{3C417F45-AD62-B24E-ADDB-2452094E5774}"/>
-    <hyperlink ref="D8" r:id="rId7" xr:uid="{055A7FF5-1139-4443-A033-FB00D12A490A}"/>
-    <hyperlink ref="D9" r:id="rId8" xr:uid="{ECCEC4A7-C0FB-204B-B77E-5D8665FD2B7C}"/>
-    <hyperlink ref="D10" r:id="rId9" xr:uid="{C57AAAAA-793D-D545-A34A-F78662E45A15}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{72B5C26E-849F-B34F-8684-398E0D547B80}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{4AE8CA51-F9AD-BF44-B2E4-2A784ED3C5BC}"/>
-    <hyperlink ref="D13" r:id="rId12" xr:uid="{A3CE98B2-674D-6C43-A93F-5393896F89BB}"/>
-    <hyperlink ref="D14" r:id="rId13" xr:uid="{B505AC96-D22F-754A-93A8-1F4DD5D185E3}"/>
-    <hyperlink ref="D15" r:id="rId14" xr:uid="{1870D29F-0933-3F49-9323-7C1B2B7EBE09}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{D1578EA7-4BEC-6745-885F-5D73DAA501C0}"/>
-    <hyperlink ref="D17" r:id="rId16" xr:uid="{AC5AF65A-2478-3D4F-9315-151689BA4C27}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="D14" r:id="rId13" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="D15" r:id="rId14" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="D16" r:id="rId15" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="D17" r:id="rId16" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>